<commit_message>
Add Plastic to the material list
Appended rather than slotted in beside the other moulded materials:
inventory is already being entered against the existing chip positions,
and reshuffling them mid-catalogue costs muscle memory for no gain.

The workbook dropdown follows. Pens already saved are untouched — the
field is optional, so anything without a material stays blank.
</commit_message>
<xml_diff>
--- a/penshow/PenShowTracker.xlsx
+++ b/penshow/PenShowTracker.xlsx
@@ -14658,7 +14658,7 @@
       <formula1>=Lists!$C$4:$C$13</formula1>
     </dataValidation>
     <dataValidation sqref="D4:D253" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Lists!$F$4:$F$8</formula1>
+      <formula1>=Lists!$F$4:$F$9</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -38717,6 +38717,11 @@
           <t>Trade</t>
         </is>
       </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Plastic</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="C10" s="4" t="inlineStr">

</xml_diff>